<commit_message>
record: add "even though" to vocab list
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Kt3M7t8oR3AYNyedAJdAM5
</commit_message>
<xml_diff>
--- a/output/vocab-list.xlsx
+++ b/output/vocab-list.xlsx
@@ -422,7 +422,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:D3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -475,6 +475,28 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>even though</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>با اینکه / هرچند</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Even though the project was difficult, we finished it on time.</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
record: add "proud" (past forms) to vocab list
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>

Claude-Session: https://claude.ai/code/session_01Kt3M7t8oR3AYNyedAJdAM5
</commit_message>
<xml_diff>
--- a/output/vocab-list.xlsx
+++ b/output/vocab-list.xlsx
@@ -422,7 +422,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:D4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -497,6 +497,28 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>proud (past: was/felt proud)</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>مغرور بودم / احساس افتخار کردم</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>I was proud of finishing the project on time.</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
record: add "incorporate" to vocab list
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>

Claude-Session: https://claude.ai/code/session_01Kt3M7t8oR3AYNyedAJdAM5
</commit_message>
<xml_diff>
--- a/output/vocab-list.xlsx
+++ b/output/vocab-list.xlsx
@@ -422,7 +422,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:D5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -519,6 +519,28 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>incorporate</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>گنجاندن / ادغام کردن</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>We incorporated solar panels into the building's design.</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
record: add "thrown off" to vocab list
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>

Claude-Session: https://claude.ai/code/session_01Kt3M7t8oR3AYNyedAJdAM5
</commit_message>
<xml_diff>
--- a/output/vocab-list.xlsx
+++ b/output/vocab-list.xlsx
@@ -422,7 +422,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:D6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -541,6 +541,28 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>thrown off</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>گیج شدن / از تمرکز خارج شدن</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>A hard question from the client threw me off during the meeting.</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add "lobes" to vocab list
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014q4dyRjtf82x138m4eq21N
</commit_message>
<xml_diff>
--- a/output/vocab-list.xlsx
+++ b/output/vocab-list.xlsx
@@ -422,7 +422,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:D4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -497,6 +497,28 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>lobes</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>لوب‌ها</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>The frontal lobes of the brain control decision-making.</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>